<commit_message>
Correct the 10/8 holds that called open POs missing.
The purchase-lines list already contained these POs. The runner dropped a line with no receipt child and reported the PO as not found. Those bills stay in Transfer AP with the real reason. UniFirst 10562 is back on batch 750 with a -$0.04 PPV because the Taxes tab cannot be edited.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/ap-run-2026-10-08/AP-run-2026-10-08.xlsx
+++ b/runs/ap-run-2026-10-08/AP-run-2026-10-08.xlsx
@@ -424,7 +424,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="88" customWidth="1" min="2" max="2"/>
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -596,7 +596,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -711,7 +711,6 @@
           <t>treyce</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -763,7 +762,6 @@
           <t>treyce</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -815,7 +813,6 @@
           <t>treyce</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -867,7 +864,6 @@
           <t>treyce</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -919,7 +915,6 @@
           <t>treyce</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -966,8 +961,6 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -1014,8 +1007,6 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -1118,8 +1109,6 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -1171,7 +1160,6 @@
           <t>shawn</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -1223,7 +1211,6 @@
           <t>treyce</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -1277,7 +1264,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Purchase order 59271 was not found. Nothing was selected.</t>
+          <t>PO 59271 is open Legacy Wire Products id 7273. Lines 01-02 are 17 ea and 33 ea 75-10-201007 at $41, received 0. No receipt on the line or in the receipts list.</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1286,7 +1273,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>1748</v>
+        <v>1763</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -1331,7 +1318,6 @@
           <t>treyce</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -1383,7 +1369,6 @@
           <t>shawn</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -1437,7 +1422,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>No open receipt matches quantity 66.0 EA. Open receipts: none.</t>
+          <t>PO 58931 receipt 24982 is 66 ea A-04421-000 for $7,171.56 and is already invoiced by bill 10491 invoice 18564 (1181-TPI). No uninvoiced qty-66 receipt.</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1446,7 +1431,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>1751</v>
+        <v>1769</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -1493,7 +1478,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>No open receipt matches quantity 38.0 EA. Open receipts: 24987 qty 62.0 EA-Each $6736.92 A-04421-000 - Fender, Drive Over.</t>
+          <t>PO 58966 has no qty-38 receipt. Receipt 24987 is 62 ea A-04421-000 and is already invoiced by bill 10554 invoice 18663. Remaining quantity 38 is not received.</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1502,7 +1487,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>1752</v>
+        <v>1770</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -1549,7 +1534,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Purchase order 59043 was not found. Nothing was selected.</t>
+          <t>PO 59043 is open TPI id 7045. Line 01 is 100 ea A-04421-000 at $108.66, received 0. No receipt recorded.</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1558,7 +1543,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>1753</v>
+        <v>1764</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -1605,7 +1590,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Purchase order 59043 was not found. Nothing was selected.</t>
+          <t>PO 59043 is open TPI id 7045. Same line, received 0. No receipt for 1 ea A-04421-000.</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1614,7 +1599,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>1754</v>
+        <v>1765</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -1661,7 +1646,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Purchase order 59061 was not found. Nothing was selected.</t>
+          <t>PO 59061 is open TPI id 7063. Line 01 is 100 ea A-04421-000 at $108.66, received 0. No receipt recorded.</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1670,7 +1655,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>1755</v>
+        <v>1766</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -1715,7 +1700,6 @@
           <t>treyce</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -1767,7 +1751,6 @@
           <t>treyce</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -1811,7 +1794,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1819,18 +1802,14 @@
           <t>treyce</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Printed sales tax is $69.22. KIMCO calculated $69.26, a $0.04 difference.</t>
-        </is>
-      </c>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>TRANSFER AP</t>
+          <t>API Agent - 10/8/26</t>
         </is>
       </c>
       <c r="K23" t="n">
-        <v>1762</v>
+        <v>1771</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -1875,7 +1854,6 @@
           <t>shawn</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
           <t>API Agent - 10/8/26</t>
@@ -1929,7 +1907,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Purchase order 59283 was not found. Nothing was selected.</t>
+          <t>PO 59283 is open Legacy Wire Products id 7285. Lines 01-02 are 27 ea and 17 ea 75-10-201007 at $41, received 0. No receipt recorded.</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1938,7 +1916,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>1760</v>
+        <v>1767</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -1985,7 +1963,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Purchase order 59303 was not found. Nothing was selected.</t>
+          <t>PO 59303 is open Legacy Wire Products id 7305. Line 02 is 10 ea 75-10-201007 at $41, received 0. No receipt recorded.</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1994,7 +1972,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>1761</v>
+        <v>1768</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -2641,7 +2619,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D39"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="4" max="4"/>

</xml_diff>